<commit_message>
Replace lt.hl7.fhir.base 0.3.0 with lt.hl7.fhir.eu 0.0.2 dependency
</commit_message>
<xml_diff>
--- a/docs/base/0.3.0/StructureDefinition-composition-lt.xlsx
+++ b/docs/base/0.3.0/StructureDefinition-composition-lt.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-15T18:57:53+02:00</t>
+    <t>2026-03-15T22:56:00+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -111,7 +111,7 @@
     <t>Base Definition</t>
   </si>
   <si>
-    <t>https://hl7.eu/fhir/StructureDefinition/CompositionEu|0.1.0-ballot</t>
+    <t>https://hl7.lt/fhir/eu/StructureDefinition/CompositionEu|0.1.0-ballot</t>
   </si>
   <si>
     <t>Abstract</t>
@@ -497,7 +497,7 @@
     <t>informationRecipient</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {http://hl7.eu/fhir/StructureDefinition/information-recipient|0.1.1}
+    <t xml:space="preserve">Extension {http://hl7.eu/fhir/StructureDefinition/information-recipient|1.2.0}
 </t>
   </si>
   <si>

</xml_diff>